<commit_message>
Auto update Pengadaan 2026-08-26 08:43:07
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-26).xlsx
@@ -1125,28 +1125,28 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>2151621112</v>
+        <v>2090003236</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>837161047</v>
+        <v>1136240668</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>774254566</v>
+        <v>1115612710.6</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1314460065</v>
+        <v>953762568</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -1505,22 +1505,22 @@
         <v>880998213</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>414252893</v>
+        <v>580813055</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>330911108</v>
+        <v>494176948</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>466745320</v>
+        <v>300185158</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -1635,25 +1635,25 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>282819298</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>141795000</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>75645612</v>
+        <v>64745634</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>141024298</v>
@@ -2871,28 +2871,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>3930</v>
+        <v>3914</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>32463190559</v>
+        <v>32401572683</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>5678297657</v>
+        <v>6143937440</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>5205203652</v>
+        <v>5698927658.6</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3567</v>
+        <v>3539</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>26784892902</v>
+        <v>26257635243</v>
       </c>
     </row>
   </sheetData>
@@ -3806,28 +3806,28 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>19502722603</v>
+        <v>19564340479</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>17085082394</v>
+        <v>17216344778</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>16328186929.4</v>
+        <v>16613057107.4</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>12034759834</v>
+        <v>12101060134</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>1</v>
@@ -3836,10 +3836,10 @@
         <v>72965295</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2417640209</v>
+        <v>2347995701</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -4320,16 +4320,16 @@
         <v>4842583639</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>1950805466</v>
+        <v>2583861466</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>1893386553</v>
+        <v>2523786553</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>11</v>
@@ -4344,10 +4344,10 @@
         <v>94888350</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2891778173</v>
+        <v>2258722173</v>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
@@ -4366,22 +4366,22 @@
         <v>24100076698</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>143</v>
+        <v>175</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>19818428400</v>
+        <v>23567530878</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>143</v>
+        <v>175</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>19351573485.03</v>
+        <v>23497213425.01</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>1773118340</v>
+        <v>2833129460</v>
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
@@ -4394,10 +4394,10 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="N32" s="10" t="n">
-        <v>4281648298</v>
+        <v>532545820</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -4596,44 +4596,44 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" s="10" t="n">
+        <v>595373450</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>273952950</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" s="10" t="n">
+        <v>153319438</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>153319438</v>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M36" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="D36" s="10" t="n">
-        <v>379426400</v>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" s="10" t="n">
-        <v>201970600</v>
-      </c>
-      <c r="G36" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H36" s="10" t="n">
-        <v>142419460</v>
-      </c>
-      <c r="I36" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J36" s="10" t="n">
-        <v>142419460</v>
-      </c>
-      <c r="K36" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L36" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M36" s="8" t="n">
-        <v>3</v>
-      </c>
       <c r="N36" s="10" t="n">
-        <v>177455800</v>
+        <v>321420500</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -6408,28 +6408,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>94656531256</v>
+        <v>94934096182</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>452</v>
+        <v>491</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>58144199754</v>
+        <v>62729602966</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>452</v>
+        <v>491</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>55726966444.43</v>
+        <v>60798776540.41</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>27417863199</v>
+        <v>28555074597</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>9</v>
@@ -6438,10 +6438,10 @@
         <v>764123653</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>36512331502</v>
+        <v>32204493216</v>
       </c>
     </row>
   </sheetData>
@@ -8047,16 +8047,16 @@
         <v>4274621970</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>3545684970</v>
+        <v>3786710370</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>2273189864.01</v>
+        <v>2513539864.01</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>1</v>
@@ -8075,10 +8075,10 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N32" s="10" t="n">
-        <v>728937000</v>
+        <v>487911600</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -10193,13 +10193,13 @@
         <v>5031291001</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>2470791364</v>
+        <v>4339950242</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>1559826000</v>
@@ -10221,10 +10221,10 @@
         </is>
       </c>
       <c r="M65" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N65" s="6" t="n">
-        <v>2560499637</v>
+        <v>691340759</v>
       </c>
     </row>
     <row r="66" ht="45" customHeight="1">
@@ -10243,13 +10243,13 @@
         <v>7626623356</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>2060207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G66" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>2058441500</v>
@@ -10271,10 +10271,10 @@
         </is>
       </c>
       <c r="M66" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N66" s="10" t="n">
-        <v>5566415556</v>
+        <v>4682415556</v>
       </c>
     </row>
     <row r="67" ht="45" customHeight="1">
@@ -10291,16 +10291,16 @@
         <v>173330864188</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>131577396506</v>
+        <v>134571580784</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>64463346946.01</v>
+        <v>64703696946.01</v>
       </c>
       <c r="I67" s="12" t="n">
         <v>127</v>
@@ -10315,10 +10315,10 @@
         <v>2980144727</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>41753467682</v>
+        <v>38759283404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>